<commit_message>
integration of vllm show good result in 161 ads
</commit_message>
<xml_diff>
--- a/data/raw/ForTest.xlsx
+++ b/data/raw/ForTest.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="RN Dimanche" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Recherche NDolo" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="RN Dimanche Good" sheetId="3" r:id="rId6"/>
-    <sheet state="hidden" name="Feuille 5" sheetId="4" r:id="rId7"/>
-    <sheet state="visible" name="Recherche NDolo Good" sheetId="5" r:id="rId8"/>
-    <sheet state="visible" name="Solidaire dans le War" sheetId="6" r:id="rId9"/>
-    <sheet state="visible" name="Offres demploi " sheetId="7" r:id="rId10"/>
+    <sheet name="RN Dimanche" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Feuille 5" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Recherche NDolo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Solidaire dans le War" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Offres demploi " sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>Date</t>
   </si>
@@ -25,7 +28,7 @@
     <t>Post</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🛑 RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -205,108 +208,10 @@
 Bonjour le warman, bjr Tata Paule bonne fête de fin d'année et merci pour tout ce que vous faites. Je suis une MC de 32ans j'ai 1 ,65(j'ai la bosse lol) pour 85kg je réside à yde je suis titulaire d'une licence en commerce actuellement je suis au chômage mais je me bat pour subvenir au besoin de ma fille. Je suis à la recherche de mon prince charmant. Il doit être propre responsable. Il doit savoir joindre l'utile à l'agréable. Mon prince si tu te reconnais dans mes écrit bien vouloir m'écrire à l'adresse suivante :amourvraietsincere02@gmail.com@gmail.com .ps les blagueurs de mbeng veillé vous abstenir svp
 -------------------- 
 DJO 17
-Bonjour tata Paule et bjr au Big katika Je suis un jeune camerounais originaire de l'ouest, âgé de 32 ans,PC résident à Douala ayant une stabilité professionnelle. Suis quelqu'un de Respectueux, ambitieux,  le sens de la famille, attentionné, comique parfois, propre, .....  Je cherche avant tout, une complice, une confidente, qui sait &lt;&lt;exactement ce qu'elle veut&gt;&gt;. Cette dernière doit être âgé entre 22 et 27 ans,, professionnellement stable, sans enfant, respectant des valeurs africaines, ambitieuse, ayant le sens de la famille,... Si ce profil te parle, n'hésite pas à laisser ton message au S_ebongue@yahoo.com
--------------------- 
-RESSE 18
-Coucou Katika, coucou tata Paule. Je traverse les atalakou car vous ne manger pas ça ! S'il vous plaît centrez ma RN au terre. Je suis fille âgée de 29 ans. Je mesure 160cm teint africain,calme, responsable et très entreprenante. Sans enfants, de la région de west et  d'expression anglaise.  Je réside a Yaoundé. Je souhaite rencontrer un homme responsable, compréhensif, aimant et qui  aime le dialogue entre 32 et 37 ans pour une relation sérieuse pouvant aboutir au mariage. Je n'accorde pas un importance capitale au physique car homme. La distance n'est pas un soucis pour moi. Si tu te vois dans ma RN, alors, merci de me contacter par ltrue9043@gmail.com 
--------------------- 
-DJO 19
-Bonjour au terre . A toi tata Paule bonjour et mes respects au warman . A 35 ans d'âge j'ai compris qu'il est temps de trouver sa meilleur amie et confidente avec qui je peux rigoler , 'aimer, faire des projets et autres .
-Je suis un jeune homme  de l'ouest avec 1 enfant  de 173cm pour 105kg sportif  résidant  à Douala.  D'après mes proches suis respectueux travailleurs et comique . Alors à toi ma futur autre moi si tu as la tranche d'âge  ]22 -30] ans  ATTENTIONNÉ et RESPECTUEUSE de préférence aimant le dialogue et bonne flatteuse écris moi à l'adresse suivante: leaderdjibril1@yahoo.fr
--------------------- 
-DJO 20
-Mes salutations cordiales à notre guide warman et Tata Paule.  Je suis un homme âgé de 40 ans, vivant à Yaoundé, pesant 82kg pour 1m80. Épanoui et équilibré dans ma vie, j'apprécie les choses simples. Passionné du travail bien fait et attaché aux valeurs traditionnelles africaines, je fais du dialogue mon leitmotiv pour construire une véritable relation.  Je recherche à travers cette plate-forme ma luciole, ma belle promise au cœur si pur pour une relation sincère et pérenne.  Si vous êtes dans la tranche de 33 à 42 ans, cultivée avec minimum bac +4, un métier stable, écrivez-moi à maluciole40@gmail.com
--------------------- 
-DJO 21
-Bonjour a tout le terre et joyeux Noël 😀 Je suis un camer de 30ans sans Mouna vivant a Yaoundé je suis grand de taille charismatique financièrement un peu stable.je recherche une girl de moins de 35ans  bio jolie posé douce financièrement stable ou mbenguiste avec ou sans enfants pour relation sérieuse pouvant aboutir au mariage.ecris moi a:love2022amour@gmail.com
--------------------- 
-DJO 22
-Bonjour le terre,Je suis un warboy vivant au KMR, fonctionnaire, de l'Ouest (NDÉ), âgé de 32, sans enfants, 1m91. Mes proches me décrivent comme quelqu'un déterminé, entreprenant, courageux. Je recherche une  wargirl agée de moins de 32ans qui veut se poser, construire et se marier. Elle devrait être au moins en fin d'études académique (de préférence stable professionnellement), stable émotionnellement, avenante, respectueuse, ouverte d'esprit, entreprenante, avoir le sens de la famille. Elle doit avoir au moins 1m65, de belles forme, le teint naturel, résider au KMR (de préférence  Yaoundé) Si tu te reconnais, écrit moi via love_agogo@yahoo.com
--------------------- 
-DJO 23
-Bonjour Tata Paul, bonjour Katika. Merci pour ce que vous faites pour la jeunesse. Je suis un jeune Camerounais de 28 ans vivant à Douala. Je me décrirais comme quelqu'un de d'abord travailleur, déterminer, ambitieux avec un grand sens des responsabilités et de la famille. De corpulence un peu au dessus de la moyenne, je mesure 1m77. Je suis à la recherche d'une perle rare, celle la encore appelée femme vertueuse que j'espère trouver ici. Elle devra avoir tout au plus 26 ans, résident au Cameroun, dans la ville de Douala de préférence. De plus, elle devra être propre et travailleuse. Je réponds à l'adresse mail : johnperry18@protonmail.com
--------------------- 
-DJO 24
-Bonjour à tous au Terre. Je suis un Warboy,de l'Ouest( Haut-Plateaux) j'ai des défauts ( esprit critique, curieux...) et des qualités ( responsable, posé, intelligent...) avec un physique agréable (1,80 mètres,79 kilos,teint chocolat, dans la quarantaine,un enfant ( je veux encore même 5) Je cherche une fille intelligente, propre, dynamique, entreprenante, respectueuse...avec 0 ou 1 enfant ayant  plus de 1,65metres entre 65 et 90 kilos  de 25 à 35 ans aimant les voyages et bilingue ( anglais et français) J'aime le réel ( donc elle doit accepter une rencontre physique réelle avant le
-début de la relation Ma chérie l'élue écrit moi à bonbeau815@gmail.com
--------------------- 
-DJO 26
-Merci KTK pour ton travail de chaque jour. Je suis un jeune camerounais résidant au kho plus précisément à Douala. En effet, je suis âgé de 29 ans, mesurant 1m82 pour 75kg et sans enfant. Deplus je suis quelqu'un de calme et réservé qui prône le dialogue et le respect mutuel entre partenaires. En outre titulaire d'un master 2 et actuellement en stage professionnel dans une entreprise de la place, je souhaite faire la rencontre d'une jeune dame âgée  de 23 ans - 30 ans possédant des valeurs familiales pour une relation sérieuse. Je réponds à l'adresse: symrejaq@gmail. com
--------------------- 
-DJO 27
-Bonjour Ktk  et le terre. Merci pour ton travail. Je suis un warboy dans la trentaine vivant à Douala. Je me débrouille au quotidien comme je peux. Je suis quelqu’un de simple et déterminé, assez réservé parfois mais avec beaucoup d’humour. Je suis à la recherche de celle là avec qui faire chemin  quelque soit les obstacles. Je recherche une personne  douce, sincère et conviviale âgée entre 21 et 25 ans vivant à Douala.  Si tu te reconnais, alors écris moi à : smoothcorasol@gmail.com PS: Pas de mère Célibataire ou de Panthère
--------------------- 
-DJO 28
-Heureuse fête de Noël à tout le terre.  Force au katika et à tata Paule pour le travail infatigable  malgré que certaines refusent de grandir dans leurs esprits.  Je recherche une femme âgée entre 25 et 32ans, CHRÉTIENNE, BIEN ÉDUQUÉE, épanouit, maternelle et veux se sentir protégée par son homme. Quant à moi, je suis un homme de 37ans, 1m80, célibataire sans enfant, travaillant à Bana depuis quelques années. Les filles vierges, compteur légèrement utilisé, anglophones, bilingues et pas abonnées aux novelas sont encouragées à l'adresse : king-priest@outlook.com
--------------------- 
-DJO 29
-Salut au big katika ,et aux membres  du terre je suis un jeune kamer résident au  237 à Douala ayant  30 ans révolu mesurant 1m79 sans mouna , je boss dans le secteur public. Je suis loyal, travailleur et très respectueux. Je recherche  cette femme qui a entre 22 et 27ans sans enfants avec les valeurs africaines respectueuse ,aimante , ouverte d'esprit, Vivant au Cameroun où ailleurs . Alors si t'es intéressée et honnête pour qu’ensemble nous construisons notre part d'avenir, je réponds à l'adresse: aviea9340@gmail.com  blagueuses s'abstenir svp🙏🏽
--------------------- 
-DJO 30
-Joyeux Noël et heureuse année 2022 aux katika et au terrerriens , je suis un jeune camerounais âgée de 32 ans, originaire de la menoua (ouest-Cameroun), célibataire et sans enfant. Jeune entrepreneur résident à Douala. teint noir, je mesure 1,77m. mon entourage me décrit comme une personne paternelle, comique. Je recherche une femme âgée minimale de 22ans et prête à s'engager pour fonder et bâtir un foyer. À toute jeune fille interressée, veille écrire à :guediaange179@gmail.com
--------------------- 
-DJO 31
-Salut à TATA Paule, au Grand WARMAN et au Terre pour cette offre de RN et tout le travail que vous faites. Je suis de l'ouest, 1,86m, 26ans, 82Kg, vivant au Kho. Je suis empathique et drôle, humble, sage avec une maturité émotionnelle/intellectuelle élevé, sachant faire la cuisine. j'ai des défauts Je cherche celle dont je serais le vent qui portera ses ailes et vice versa. Elle doit avoir une 👍🏾 moralité, croyante, soumise, travailleuse, cultivé, attentionné, avec Âge (19-24), (Taille:M 1,65-1,85), Poids &lt;82Kg), NB: 👩👧👧 et 👨👩👧 ne sont pas concernés. sapiovalentinamour@yahoo.com
--------------------- 
-DJO 32
-Bonjour Big Katika.J'aimerai par mon annonce rencontrer ma déesse. Suis âgé de 29 ans (1m89 pour 78kg mince) célibataire, sans enfants. J'ai Master, suis professionnellement actif et réside à Yaoundé. J'aime faire mon sport hebdomadaire, la lecture, voyages et aussi  cuisiner. Bref, je me décrirai comme quelqu'un de  posé et attentionné. Je recherche ma déesse âgée minimum de 21 ans et +, qui désire s'engager dans une relation franche, sincère et durable.
-Ma binôme doit avoir sa tête sur ses épaules. En gros je ne saurais là dessinée à  travers un clavier. Tu te sens prête ? alors écris à krysbyme@gmail.com
--------------------- 
-DJO 33
-Bonjour warman, Jeune camerounais de 29 ans, 1m80  pour 85kg, Centre, vivant à Yaoundé, célibataire sans enfants, je suis médecin exerçant à Yaoundé et financièrement stable, calme, ambitieux, bosseur, posé et très drôle! Je cherche une fille vivant à yde, âgée de 22 a 27ans, financièrement stable ou en fin de formation dans une école à emploi direct, célibataire sans enfant, faisant entre 1m60 et 1m75, de corpulence moyenne avec les formes généreuses à l'africaine et naturellement jolie! posée, propre, simple, attentionnée et joviale! J'aime les filles qui savent faire la cuisine!  secretamour87@yahoo.com 
-________________________________
-🛑 Si Vous aussi vous souhaitez faire passer votre annonce Cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
-__________________________________ 
-🔴 Pour faire passer votre publicité au terre, Contactez nous via WhatsApp pour la procédure et les modalités en cliquant sur: 
-https://wa.me/+237696493067
-Votre publication sera faite:
-🟡Sur la page facebook du warman + de 250 000 abonnés
-🟡Dans son groupe facebook + de 150 000 membres
-🟡Dans le groupe Telegram du warman +de 8 300 membres
-🟡Dans le groupe Facebook des Wargirls + de 50 000 membres
-____________________________________________________________________
-🛑 Tous les fonds récoltés pour les annonces (publicités ou recherche ndolo) sont destinés au fonctionnement de l’association : Solidaire dans le War 
-________________________________ 
-🛑 En savoir plus sur l’association solidaire dans le war : 
-https://www.warmanduterre.com/solidairedanslewar
-___________________________________________________________________ 
-🛑 Pour lire les Témoignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publiés-sur-la-page-warman-du-terre</t>
+Bonjour tata Paule et bjr au Big katika Je suis un jeune camerounais originaire de l'ouest, âgé de 32 ans,PC résident à Douala ayant une stabilité professionnelle. Suis quelqu'un de Respectueux, ambitieux,  le sens de la famille, attentionné, comique parfois, propre, .....  Je cherche avant tout, une complice, une confidente, qui sait &lt;&lt;exactement ce qu'elle veut&gt;&gt;. Cette dernière doit être âgé e</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
-Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
-_________________________
-Bonjour au  grand frère Warman et à tata Paule! Je tiens à vous remercier pour le grand travail que vous abattez au sein de la communauté. Je suis une  camerounaise âgé de 35ans résident au Canada. 
-Célibataire sans enfant, en début de carrière, pèse 70kg/ 1.70. J'attends souvent dire de moi que je suis  respectueuse, douce et travailleuse. 
-J'ai décidé de faire cette annonce à la recherche de mon mâle dominant avec qui on doit fonder une famille solide. 
-Avoir entre 35-42ans , resident au Canada sans enfant ou un au trop. Il doit mesurer 1.72 et plus, etre travailleur, respectueux et le sens de l'humour... 
-A toi qui lis ceci si tu remplis les critères et aimerait en savoir plus je t'attends chaleureusement 
-👉👉👉 
-Amouradeux202201@yahoo.com
-_______________________
-⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
-🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
-____________________________
-👉🏾 💚❤️💛 Tu cherches celle la qui va te suilever jusqu’au ciel?  jusqu’à Dieu va encadrer votre ndolo et vous donner sa chaise là où il faut, par la reine du règne et la roi de gloire ??
-Ne cherche plus, fais juste les recherches ndolo, rédige ton annonce de recherche du partenaire idéal pour toi et nous posterons ton annonce
-Contactez nous via WhatsApp pour la procédure et les modalités en cliquant sur: 
-   https://wa.me/+237696493067
-  Votre publication sera faite:
-    🟡Sur la page facebook du warman + de 250 000 abonnés
-     🟡Dans son groupe facebook + de 150 000 membres
-      🟡Dans le groupe Telegram du warman +de 8 000 membres
-      🟡Dans le groupe Facebook des Wargirls + de 50 000 membres
-  ________________________________ 
-🟤 En savoir plus sur l’association solidaire dans le war : 
-         https://www.warmanduterre.com/solidairedanslewar
-         ________________________________ 
-🟢 Pour lire les Témoignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publiés-sur-la-page-warman-du-terre
-        ____________________________ 
-🔴 Nouveau Le Terre est sur télégram :
-           https://t.me/WarmanduTerreATerre</t>
-  </si>
-  <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 💚❤️💛 RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -495,7 +400,7 @@
 ￼Dans le groupe Facebook des Wargirls + de 50 000 membres</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -691,11 +596,10 @@
 Bonjour au terre et warman! Je suis une camerounaise vivant au Cameroun, j'ai 26ans et je mesure un mesure 1,70m de taille ayant un enfant. Je suis étudiante et je fais aussi de petits boulots. Je suis à la recherche de mon âme sœur, beau, séduisant, doux, respectueux. Âgé de 30 à 45ans de préférence basé au Cameroun ou alors hors du Cameroun et ayant des visions de former une bonne famille. Je suis joignable à l'adresse : lydiebeyene@gmail.com
 ________________________________
 🛑 Si Vous aussi vous souhaitez faire passer votre annonce Cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
-__________________________________ 
-🔴 Pour faire passer votre publicité au terre, Contactez nous via WhatsApp pour la procédure et les modalités en cliquant sur: </t>
+__________</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
    RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -888,7 +792,7 @@
 🛑 Pour lire les Témoignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publiés-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -1047,7 +951,7 @@
 🟡Dans le groupe Telegram du warman +de 8 300 membres</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
    RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -1229,7 +1133,7 @@
 ________________________________</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
  🔴 RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -1404,7 +1308,7 @@
 🛑 Pour lire les Témoignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publiés-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
  RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -1600,7 +1504,7 @@
 https://www.warmanduterre.com/solidairedanslewar</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
   RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -1795,7 +1699,7 @@
   https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
   RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -1983,42 +1887,10 @@
 Bonjour le terre merci tata Paule et au warman pour cette initiative. Je suis une femme âgée de 30 ans à la recherche de sa moitié j'ai un enfant, residente à Yaoundé. je suis originaire de l'ouest financièrement stable; les personnes de mon entourage me décrivent comme une personne réservée, aimante, ayant un grand cœur et le sens de la famille.  Je suis à la recherche d'un homme ayant au moins 30 ans, il doit être financièrement stable, responsable, qui veut déjà fonder sa famille. Mon apollon, mon paracétamol si tu te reconnais dans cette description n'hésite pas à m'écrire: Ndolokr@gmail.com
 -------------------- 
 RESSE 24
-Bonjour tata paule,bonjour warman,bjr le terre. Je suis une femme de 30 ans sans enfants,de teint noir ,ronde avec des formes faisant un 1 m 57.je vis a douala.je fais dans la vente de vetements dans un marche de la place.je suis une personne sincere,battante et comprehensive.je recherche un homme age entre 31 et 35 ans sans enfant et stable financierement avec qui on pourra vivre une belle histoire damour et fonder une famille.vivre aupre dun homme qui nous aime et qu on aime est plus paisible que de vivre seule.ecris moi a ladresse etoile.or07@gmail.com
--------------------- 
-RESSE 25
-Bonjour .camerounaise de 31ans, 1m69 sans enfants originaire du Littoral). réside à Douala où je bosse. Pas assez de possibilité de faire de rencontres vu mn côté casanier aussi . (femme 🙂)calme, posée, mature sachant ce qu'elle veut dans la vie.je viens donc par ce canal espérant trouver ma moitié quelqu'un ayant des même visions que moi âgée entre 33et 43ans de bonne moralité, financièrement stable et maximum 1 enfant.celui-ci devra résider de préférence à Douala.Mais je reste ouverte aux autres car ''on ne sait jamais''.Les jongleurs prière de vous abstenir !!! nachamour@yahoo.com
--------------------- 
-RESSE 26
-je suis une fille début de la trentaine sans enfants, benjamine d'une fratrie de plusieurs enfants, on dit de moi que je suis sympa ,joviale ,pleinede vie et capricieuse peut-être du au fait que je sois dernière née et que je sois encore la seule vivant avec mes parents lol. Je suis en activité ds le  business de ces derniers et je souhaiterai rencontrer un homme âgé entre 35 et 43 ans avec max un enfant , qui bosse , la situation géographique n'en serait en rien un obstacle s'il est sincère ,loyal voulant une relation pouvant aboutir au mariage M'écrire via ndolocamer21@gmail.com
--------------------- 
-RESSE 27
-Bonjour au TERRE. Jeune Camerounaise de 24ans, célibataire sans enfants au teint choco(nb:1m67 pour 62kg), je boss et je suis parallèlement en fin de formation à Yaoundé, ville dans laquelle je réside. Très souvent, je suis qualifiée de Réservée,( jusqu'à ce que je me sente en sécurité😅).Aussi Respectueuse qu'attentionnée, je tiens à nos valeurs Chrétiennes et culturelles. Alors, à toi mon bien aimé, je sais que tu es un homme ATTENTIONNÉ, respectueux,  âgé entre 24 et 35 ans sans enfants, qui connait la valeur d'une épouse, vivant près de moi ou peu importebemylove237@gmail.com
--------------------- 
-RESSE 28 
-Bonjour Katika et Tata Paule. Je suis une dame de 27ans vivant au Cameroun de teint caramel mesurant 1m60 pour 73kg  originaire du Littoral (Bassa'a) agréable a admirer, séropositive sans enfant.Titulaire d'une licence professionnelle je me débrouille dans tous ce qui est digne.
-Je suis responsable,Ambitieuse, travailleuse et Ouverte,passionnée de cuisine,voyage et Romance.Je recherche un homme âgé de 30-40ans responsable, intègre,sage, ambitieux et tolérant avec ou sans enfant.Je prône le dialogue, le respect, la confiance et le partage. Si tu te reconnais dans ma description je serais ravie de te lire: orpheelove04@gmail.com Longue vie au TERRE
--------------------- 
-RESSE 29
-Bonjour  le terre  je suis une camerounaise de l'ouest  je reside a douala âgé de 33 ans MC  d'une fille   je fais 1m60  pour 70k. Je me bat au quotidien pour m'occuper de ma famille  mon entourage me definit comme une personne généreuse  ouverte    battante    et ambitieuse  j'aimerais donc la rencontre d'un homme donc l âge varie 35-47 ans non fumeur  ayant le sens du vivre ensemble      l'amour vraie se base sur la confiance le respect le dialogue le respect  le pardon et lhumilite. écris moi à l'adresse mimiamour86@gmail.com
--------------------- 
-RESSE 30
-Salut le terre👋🏾 Jeune camerounaise de 25 ans célibataire sans enfants, originaire du haut - nkam, étudiante en santé vivant a Douala, travailleuse, ambitieuse respectueuses et douce. Je mesure 1,68m pour 70kg de teint chocolat.  Recherche un homme âgé de 28 à 40 ans grand de taille, ambitieux, travailleurs, respectueux et surtout doux et protecteur avec sa moitié.   Si tu souhaites te poser et construire une relation qui pourra aboutir au mariage, laisse moi un mail👇🏽  sucredorge207@gmail.com
-________________________________
-🛑 Si Vous aussi vous souhaitez faire passer votre annonce Cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
-__________________________________ 
-🛑 Vous souhaitez présenter votre page Facebook, chaîne YouTube, business ou entreprise par vidéo, ou via une publication individuelle et accompagné de photos ?  
-Sur la page Facebook du Warman ou dans le groupe Facebook Warman du terre  Ecrivez au +237 696 49 30 67 via whatsapp pour les modalités de paiement
-ou en cliquant sur https://wa.me/+237696493067
-____________________________________________________________________
-🛑 Tous les fonds récoltés pour les annonces (publicités ou recherche ndolo) sont destinés au fonctionnement de l’association : Solidaire dans le War 
-________________________________ 
-🛑 En savoir plus sur l’association solidaire dans le war : 
-https://www.warmanduterre.com/solidairedanslewar
-___________________________________________________________________ 
-🛑 Pour lire les Témoignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publiés-sur-la-page-warman-du-terre</t>
+Bonjour tata paule,</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
   RECHERCHE NDOLO 100% KMER ( Page 1 sur 2 )
      ( Chaque Dimanche Matin )
 Si vous souhaitez faire passer une annonce sur la page, cliquez sur ce lien pour demander les modalités : https://wa.me/+237696493067
@@ -2202,22 +2074,10 @@
 RESSE 26
 Bonjour big, stp centre mon annonce si au terre. Je suis une jeune demoiselle âgée de 26ans sans enfant, originaire de l'ouest et résidant à Douala. Par ce biais je souhaiterai rencontrer cette homme qui saura être un complice, protecteur, un partenaire.Quelqu'un de responsable, bosseur, ambitieux, attentionné ouvert... Qui sait valoriser sa chérie. Pour ce qui me concerne, je me décrirai comme une personne plutôt calme, battante,posée ayant le sens de la famille... Avec des défauts également. Si tu souhaites en savoir plus beautylonnie@gmail.com
 ________________________________
-🛑 Si Vous aussi vous souhaitez faire passer votre annonce Cliquez sur ce lien pour demander les modalités : https://wa.me/message/7N3B53BQMTC7O1
-__________________________________ 
-🛑 Vous souhaitez présenter votre page Facebook, chaîne YouTube, business ou entreprise par vidéo, ou via une publication individuelle et accompagné de photos ?  
-Sur la page Facebook du Warman ou dans le groupe Facebook Warman du terre
-Ecrivez au +237 696 49 30 67 via whatsapp pour les modalités de paiement
-ou en cliquant sur https://wa.me/+237696493067
-____________________________________________________________________
-🛑 Tous les fonds récoltés pour les annonces (publicités ou recherche ndolo) sont destinés au fonctionnement de l’association : Solidaire dans le War 
-________________________________ 
-🛑 En savoir plus sur l’association solidaire dans le war : 
-https://www.warmanduterre.com/solidairedanslewar
-___________________________________________________________________ 
-🛑 Pour lire les Témoignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publiés-sur-la-page-warman-du-terre</t>
+🛑 Si Vous aussi vous souhaitez faire passer votre annonce Cliquez sur ce lien pour demander les modalités : https://w</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT D' ALLEMAGNE 🇩🇪
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT D' ALLEMAGNE 🇩🇪
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2244,7 +2104,40 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇫🇷
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
+_________________________
+Bonjour au  grand frère Warman et à tata Paule! Je tiens à vous remercier pour le grand travail que vous abattez au sein de la communauté. Je suis une  camerounaise âgé de 35ans résident au Canada. 
+Célibataire sans enfant, en début de carrière, pèse 70kg/ 1.70. J'attends souvent dire de moi que je suis  respectueuse, douce et travailleuse. 
+J'ai décidé de faire cette annonce à la recherche de mon mâle dominant avec qui on doit fonder une famille solide. 
+Avoir entre 35-42ans , resident au Canada sans enfant ou un au trop. Il doit mesurer 1.72 et plus, etre travailleur, respectueux et le sens de l'humour... 
+A toi qui lis ceci si tu remplis les critères et aimerait en savoir plus je t'attends chaleureusement 
+👉👉👉 
+Amouradeux202201@yahoo.com
+_______________________
+⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
+🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
+____________________________
+👉🏾 💚❤️💛 Tu cherches celle la qui va te suilever jusqu’au ciel?  jusqu’à Dieu va encadrer votre ndolo et vous donner sa chaise là où il faut, par la reine du règne et la roi de gloire ??
+Ne cherche plus, fais juste les recherches ndolo, rédige ton annonce de recherche du partenaire idéal pour toi et nous posterons ton annonce
+Contactez nous via WhatsApp pour la procédure et les modalités en cliquant sur: 
+   https://wa.me/+237696493067
+  Votre publication sera faite:
+    🟡Sur la page facebook du warman + de 250 000 abonnés
+     🟡Dans son groupe facebook + de 150 000 membres
+      🟡Dans le groupe Telegram du warman +de 8 000 membres
+      🟡Dans le groupe Facebook des Wargirls + de 50 000 membres
+  ________________________________ 
+🟤 En savoir plus sur l’association solidaire dans le war : 
+         https://www.warmanduterre.com/solidairedanslewar
+         ________________________________ 
+🟢 Pour lire les Témoignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publiés-sur-la-page-warman-du-terre
+        ____________________________ 
+🔴 Nouveau Le Terre est sur télégram :
+           https://t.me/WarmanduTerreATerre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇫🇷
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 _________________________
 Bonjour warman et au terre. Qui suis-je? Une femme de 39 ans ( déjà!) vivant à Paris, stable professionnellement et maman d'un garçon de bientôt 4 ans.
@@ -2284,7 +2177,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 _________________________
 Bonsoir warman merci pour le travail exceptionnel que vous faite dans la communauté camerounaise. Je suis une dame âgée de 38 ans mère célibataire de 3 enfants de l'ouest Cameroun vivant au Canada. Respectueuse,gentille,responsable et qui aime la vie.je suis travailleuse courageuse persévérante et je projette dans un avenir mon sens d'ecoute et d'auto critique m'aide à m'améliorer positivement sur tout les plans de ma vie.jaimerais faire la rencontre d'un homme futur époux aimant responsable ayant des valeurs axée sur le respect la vérité l'amour la communication et les valeurs ancestrales.jaime danser voyager faire des sorties en couple et en famille aller au cinéma soirée romantique .mon coeur si tu es cet homme que je recherche honnête sincère travailleur vrai et ayant le sens de la famille âgée entre 40 et 55 ans, avec ou sans enfants, résident au Canada et pense avoir trouvé celle qu'il te faut alors communique avec moi c'est avec plaisir que je te lirait tu peux m'écrire a
@@ -2313,7 +2206,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 _________________________
 Bonjour Warman,
@@ -2346,7 +2239,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 _________________________
 Bonsoir tonton Warman, bonsoir tâta Paule et salutation le terre.
@@ -2382,7 +2275,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 _________________________
 bonsoir warman
@@ -2418,7 +2311,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT D' ALLEMAGNE 🇩🇪
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT D' ALLEMAGNE 🇩🇪
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 _________________________
 Bonsoir Warman,
@@ -2462,7 +2355,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DES USA 🇺🇲
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DES USA 🇺🇲
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 Bonjour Warman, bonjour Tata Paule, mes salutations au terre. 
 Je suis âgée de 32 ans et je réside aux États-Unis dans le Maryland. Je suis disposée à déménager si la relation devient sérieuse. Je suis originaire de l'ouest Cameroun avec un physique digne d'une reine mère. Je suis très ronde avec tout ce qu'il faut là où il faut. J'ai 1m63 et je suis de teint noir. Je suis titulaire d'un Master en marketing et je suis financièrement stable. Je suis attentionnée, honnête et généreuse mais aussi impatiente, timide et capricieuse🙈. Etant donné que je ne sors pas beaucoup, surtout en ce moment de crise sanitaire, mes chances de rencontrer quelqu'un sont très limitées. Je viens donc ici en espérant trouver un homme vivant en Europe, au Canada ou aux États-Unis, dont l'âge se situe entre 32 et 42 ans. Il doit avoir un niveau d'études supérieures, un emploi stable, une situation régulière et le désir de fonder une famille dans un avenir très proche. J'aimerais qu'il soit attentionné, généreux, patient, ambitieux et non fumeur.Je suis attirée par les hommes faisant au moins 1m80, costauds, avec une apparence soignée. Je veux être celle qui lui fera son 1er enfant. 
@@ -2491,7 +2384,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE  🇨🇵
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE  🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2524,7 +2417,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE  🇨🇵
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE  🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2557,7 +2450,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA  🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA  🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2592,7 +2485,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE BELGIQUE 🇧🇪
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE BELGIQUE 🇧🇪
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2627,7 +2520,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CAMEROUN 🇨🇲
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CAMEROUN 🇨🇲
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2668,7 +2561,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2704,7 +2597,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2739,7 +2632,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2776,7 +2669,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2810,10 +2703,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>05/11/0201</t>
-  </si>
-  <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE BELGIQUE 🇧🇪
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE BELGIQUE 🇧🇪
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2858,7 +2748,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CAMEROUN 🇨🇲
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CAMEROUN 🇨🇲
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2899,7 +2789,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2943,7 +2833,7 @@
 🟤 En savoir plus sur l’association solidaire dans le war :</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CAMEROUN 🇨🇲
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CAMEROUN 🇨🇲
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -2980,7 +2870,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DES USA 🇺🇸
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DES USA 🇺🇸
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3015,7 +2905,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE SUISSE 🇨🇭
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE SUISSE 🇨🇭
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3048,7 +2938,7 @@
            https://t.me/WarmanduTerreATerre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT D'ALLEMAGNE 🇩🇪
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT D'ALLEMAGNE 🇩🇪
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3109,7 +2999,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3136,7 +3026,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3166,7 +3056,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3192,7 +3082,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3219,7 +3109,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3245,7 +3135,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦 
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦 
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3275,7 +3165,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER 🇨🇲 VENANT D'ALLEMAGNE 🇩🇪
+    <t xml:space="preserve">💚❤️💛 SPECIAL RECHERCHE NDOLO 100% KMER 🇨🇲 VENANT D'ALLEMAGNE 🇩🇪
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 ⬜ Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3303,7 +3193,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DE FRANCE 🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3331,7 +3221,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU FRANCE 🇨🇵
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU FRANCE 🇨🇵
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3358,7 +3248,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3388,7 +3278,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER 🇨🇲
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER 🇨🇲
                VENANT D’ ITALIE 🇮🇹
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
@@ -3417,7 +3307,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -3446,7 +3336,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER
                VENANT DE FRANCE
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
@@ -3480,7 +3370,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER
                VENANT DE FRANCE
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
@@ -3514,7 +3404,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER
                    VENANT DE FRANCE
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé !
@@ -3543,7 +3433,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER
                    VENANT DE FRANCE
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé !
@@ -3572,7 +3462,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER
                    VENANT DU CAMEROUN
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé !
@@ -3600,7 +3490,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🔴PARTICIPATION 
+    <t xml:space="preserve">🔴PARTICIPATION 
 🔺Résumé : Une cagnotte a été ouverte le 5 décembre en faveur des orphelins. vos contributions sont attendus SVP.
 Ici https://www.facebook.com/groups/warmanduterre.legroupe/permalink/660972284907044/
 ⬜NOM: Le bon berger
@@ -3642,7 +3532,7 @@
 _________________</t>
   </si>
   <si>
-    <t>Bonsoir Chers membres du terre, comme vous le savez nous organisons chaque fin d’année une cagnotte pour les mounas défavorisés du kho afin de leur donner un peu de joie au cœur.
+    <t xml:space="preserve">Bonsoir Chers membres du terre, comme vous le savez nous organisons chaque fin d’année une cagnotte pour les mounas défavorisés du kho afin de leur donner un peu de joie au cœur.
 Suite à la descente de Tata Paule le 4 décembre dans un orphelinat à Nkoabang  sis à Yaoundé, j’ai décidé via mon association caritative Solidaire dans le War de leur venir en aide, et je compte sur votre grande générosité pour nous soutenir cette initiative comme vous l’avez déjà fait plusieurs fois.  
 ___________________
 Voici les moyens de contribution :
@@ -3664,7 +3554,7 @@
 _________________</t>
   </si>
   <si>
-    <t>PARTICIPONS
+    <t xml:space="preserve">PARTICIPONS
 Rebonjour 
 Je  suis la jeune dame de 40ans qui
 A contactée le grand war
@@ -3677,7 +3567,7 @@
 --</t>
   </si>
   <si>
-    <t>SUITE  DE LA RESSÉ  AGRESSEE PAR SON ONCLE ET SON  GAR HEIN
+    <t xml:space="preserve">SUITE  DE LA RESSÉ  AGRESSEE PAR SON ONCLE ET SON  GAR HEIN
 Bonjour tonton  warman depuis la dernière fois que nous avons causer grâce à l'aide que la grande famille du terre m'avais apporter j'ai réussi a fuir mon ex et quitté Douala pour le village.
 De la j'ai changer le numéro pour ne plus avoir a faire a lui.
 Les choses ne se sont pas passer comme j'avais souhaitez , et je ne voulais plus te dérangé et tout le terre car vous aviez vraiment beaucoup fait pour moi vous avez fait pour moi ce que nul n'avais fait avant  une fois de plus grand merci a toi tonton warman 
@@ -3698,7 +3588,7 @@
 ------</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -3815,7 +3705,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -3904,7 +3794,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -4163,7 +4053,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -4415,7 +4305,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -4689,7 +4579,7 @@
 P.S : Nous ne recevons que les offres d’emploi, N’ENVOYEZ NI VOS CV, NI VOS DEMANDES D’EMPLOI.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -4853,7 +4743,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -5086,7 +4976,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -5202,7 +5092,7 @@
 🔴 Envoyez vos OFFRES D’EMPLOI via WhatsApp en cliquant sur : https://wa.me/+237696493067</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -5463,7 +5353,7 @@
 Attention : Nous déclinons toute responsabilité en cas de mésentente entre l’employeur et vous. C’est à vous les postulants de faire attention aux dérives (demande de frais de dossier, abus ...)</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -5688,7 +5578,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -5839,7 +5729,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>WARMAN DU TERRE A TERRE 🇨🇲:
+    <t xml:space="preserve">WARMAN DU TERRE A TERRE 🇨🇲:
 🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
@@ -5934,7 +5824,7 @@
 Warman du terre.</t>
   </si>
   <si>
-    <t>🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
+    <t xml:space="preserve">🛑 SPECIAL RECHERCHE NDOLO 100% KMER🇨🇲 VENANT DU CANADA 🇨🇦
 Si vous aussi souhaitez faire passer une annonce spéciale Recherche Ndolo sur la page, cliquez sur ce lien pour demander les modalités: https://wa.me/+237696493067
 ⚠️ Attention le numéro pour s'enregistrer a changé les frais de publication aussi!
 🟡 Nouveau Le Terre est sur télégram : https://t.me/WarmanduTerreATerre
@@ -5961,7 +5851,7 @@
 🛑 Pour lire les Te‌moignages Ndolo allez sur : https://www.warmanduterre.com/post/temoignages-des-recherches-ndolo-publie‌s-sur-la-page-warman-du-terre</t>
   </si>
   <si>
-    <t>🔴 OFFRES D’EMPLOI
+    <t xml:space="preserve">🔴 OFFRES D’EMPLOI
 VOUS RECRUTEZ ? VOUS RECHERCHEZ DES : Ingénieurs, Architectes, Informaticiens, Enseignants, Commis, Réceptionnistes, Hôtesses, Vendeurs, Nounous, Chauffeurs, Cadres, Secrétaires, Médecin, Infirmiers, Ménagères, Cuisiniers…
 🔴 Envoyez vos offres d’emploi via WhatsApp en cliquant sur : https://wa.me/+237696493067
 L’offre d’emploi doit contenir :
@@ -6025,15 +5915,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
+      <sz val="10.000000"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -6054,69 +5944,336 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -6173,7 +6330,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -6199,7 +6356,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -6276,7 +6433,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -6306,17 +6463,19 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="12.88"/>
+    <col customWidth="1" min="2" max="2" width="12.880000000000001"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6329,44 +6488,99 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>44556.0</v>
+        <v>44556</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2"/>
+      <c r="A3" s="2">
+        <v>44549</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2"/>
+      <c r="A4" s="2">
+        <v>44542</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2"/>
+      <c r="A5" s="2">
+        <v>44535</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2"/>
+      <c r="A6" s="2">
+        <v>44528</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2"/>
+      <c r="A7" s="2">
+        <v>44521</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2"/>
+      <c r="A8" s="2">
+        <v>44514</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2"/>
+      <c r="A9" s="2">
+        <v>44507</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2"/>
+      <c r="A10" s="2">
+        <v>44499</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2">
+        <v>44493</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2"/>
+      <c r="A12" s="2">
+        <v>44486</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2"/>
+      <c r="A13" s="2">
+        <v>44485</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2"/>
@@ -6437,6 +6651,9 @@
     <row r="36">
       <c r="A36" s="2"/>
     </row>
+    <row r="37">
+      <c r="A37" s="2"/>
+    </row>
     <row r="38">
       <c r="A38" s="2"/>
     </row>
@@ -6449,17 +6666,66 @@
     <row r="41">
       <c r="A41" s="2"/>
     </row>
+    <row r="42">
+      <c r="A42" s="2"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2"/>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetData/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
@@ -6471,144 +6737,343 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>44554.0</v>
+        <v>44554</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2"/>
+      <c r="A3" s="2">
+        <v>44547</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2"/>
+      <c r="A4" s="2">
+        <v>44543</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2"/>
+      <c r="A5" s="4">
+        <v>44543</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2"/>
+      <c r="A6" s="2">
+        <v>44540</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2"/>
+      <c r="A7" s="2">
+        <v>44540</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2"/>
+      <c r="A8" s="2">
+        <v>44534</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2"/>
+      <c r="A9" s="2">
+        <v>44534</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2"/>
+      <c r="A10" s="2">
+        <v>44533</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2">
+        <v>44524</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2"/>
+      <c r="A12" s="2">
+        <v>44518</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2"/>
+      <c r="A13" s="2">
+        <v>44517</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2"/>
+      <c r="A14" s="2">
+        <v>44516</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2"/>
+      <c r="A15" s="2">
+        <v>44509</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2"/>
+      <c r="A16" s="2">
+        <v>44509</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2"/>
+      <c r="A17" s="2">
+        <v>44505</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2"/>
+      <c r="A18" s="2">
+        <v>44505</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2"/>
+      <c r="A19" s="2">
+        <v>44327</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2"/>
+      <c r="A20" s="2">
+        <v>44504</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2"/>
+      <c r="A21" s="2">
+        <v>44504</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2"/>
+      <c r="A22" s="2">
+        <v>44503</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2"/>
+      <c r="A23" s="2">
+        <v>44500</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2"/>
+      <c r="A24" s="4">
+        <v>44500</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2"/>
+      <c r="A25" s="4">
+        <v>44496</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2"/>
+      <c r="A26" s="2">
+        <v>44496</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2"/>
+      <c r="A27" s="2">
+        <v>44495</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2"/>
+      <c r="A28" s="2">
+        <v>44494</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2"/>
+      <c r="A29" s="2">
+        <v>44493</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2"/>
+      <c r="A30" s="2">
+        <v>44492</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="2"/>
+      <c r="A31" s="2">
+        <v>44491</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2"/>
+      <c r="A32" s="2">
+        <v>44488</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2"/>
+      <c r="A33" s="2">
+        <v>44485</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2"/>
+      <c r="A34" s="4">
+        <v>44484</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="2"/>
+      <c r="A35" s="2">
+        <v>44483</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2"/>
+      <c r="A36" s="2">
+        <v>44481</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="2"/>
+      <c r="A37" s="2">
+        <v>44480</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2"/>
+      <c r="A38" s="2">
+        <v>44477</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="2"/>
+      <c r="A39" s="2">
+        <v>44476</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2"/>
+      <c r="A40" s="2">
+        <v>44476</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2"/>
+      <c r="A41" s="2">
+        <v>44474</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2"/>
+      <c r="A42" s="2">
+        <v>44474</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="2"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2"/>
+      <c r="A43" s="4">
+        <v>44474</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2"/>
     </row>
-    <row r="46">
-      <c r="A46" s="2"/>
-    </row>
     <row r="47">
       <c r="A47" s="2"/>
     </row>
@@ -6888,6 +7353,9 @@
     <row r="139">
       <c r="A139" s="2"/>
     </row>
+    <row r="140">
+      <c r="A140" s="2"/>
+    </row>
     <row r="141">
       <c r="A141" s="2"/>
     </row>
@@ -7029,9 +7497,6 @@
     <row r="187">
       <c r="A187" s="2"/>
     </row>
-    <row r="188">
-      <c r="A188" s="2"/>
-    </row>
     <row r="189">
       <c r="A189" s="2"/>
     </row>
@@ -7083,1408 +7548,339 @@
     <row r="205">
       <c r="A205" s="2"/>
     </row>
+    <row r="206">
+      <c r="A206" s="2"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="2"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="2"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="2"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="2"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="2"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="2"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="2"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="2"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="2"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="2"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="2"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="2"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="2"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="2"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="2"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="2"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="2"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="2"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="2"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="2"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="2"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="2"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="2"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="2"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="2"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="2"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="2"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="2"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="2"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="2"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="2"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="2"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="2"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="2"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="2"/>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="2" max="2" width="12.88"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
-        <v>44556.0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>44549.0</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>44542.0</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>44535.0</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>44528.0</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>44521.0</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>44514.0</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>44507.0</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>44499.0</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2">
-        <v>44493.0</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2">
-        <v>44486.0</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2">
-        <v>44485.0</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2"/>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <sheetData/>
-  <drawing r:id="rId1"/>
+  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2">
+        <v>44544</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>44535</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>44514</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>44494</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2"/>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
-        <v>44554.0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>44547.0</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>44543.0</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4">
-        <v>44543.0</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>44540.0</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>44540.0</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>44534.0</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>44534.0</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>44533.0</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2">
-        <v>44524.0</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2">
-        <v>44518.0</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2">
-        <v>44517.0</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2">
-        <v>44516.0</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2">
-        <v>44509.0</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2">
-        <v>44509.0</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2">
-        <v>44505.0</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2">
-        <v>44505.0</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2">
-        <v>44504.0</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2">
-        <v>44504.0</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2">
-        <v>44503.0</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2">
-        <v>44500.0</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4">
-        <v>44500.0</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4">
-        <v>44496.0</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2">
-        <v>44496.0</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2">
-        <v>44495.0</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2">
-        <v>44494.0</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2">
-        <v>44493.0</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2">
-        <v>44492.0</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2">
-        <v>44491.0</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2">
-        <v>44488.0</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2">
-        <v>44485.0</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4">
-        <v>44484.0</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2">
-        <v>44483.0</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2">
-        <v>44481.0</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2">
-        <v>44480.0</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2">
-        <v>44477.0</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2">
-        <v>44476.0</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2">
-        <v>44476.0</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2">
-        <v>44474.0</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2">
-        <v>44474.0</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4">
-        <v>44474.0</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="2"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="2"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="2"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="2"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="2"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="2"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="2"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="2"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="2"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="2"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="2"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="2"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="2"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="2"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="2"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="2"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="2"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="2"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="2"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="2"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="2"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="2"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="2"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="2"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="2"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="2"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="2"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="2"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="2"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="2"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="2"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="2"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="2"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="2"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="2"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="2"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="2"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="2"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="2"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="2"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="2"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="2"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="2"/>
-    </row>
-    <row r="123">
-      <c r="A123" s="2"/>
-    </row>
-    <row r="124">
-      <c r="A124" s="2"/>
-    </row>
-    <row r="125">
-      <c r="A125" s="2"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="2"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="2"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="2"/>
-    </row>
-    <row r="129">
-      <c r="A129" s="2"/>
-    </row>
-    <row r="130">
-      <c r="A130" s="2"/>
-    </row>
-    <row r="131">
-      <c r="A131" s="2"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="2"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="2"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="2"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="2"/>
-    </row>
-    <row r="136">
-      <c r="A136" s="2"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="2"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="2"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="2"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="2"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="2"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="2"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="2"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="2"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="2"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="2"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="2"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="2"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="2"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="2"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="2"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="2"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="2"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="2"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="2"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="2"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="2"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="2"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="2"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="2"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="2"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="2"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="2"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="2"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="2"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="2"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="2"/>
-    </row>
-    <row r="168">
-      <c r="A168" s="2"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="2"/>
-    </row>
-    <row r="170">
-      <c r="A170" s="2"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="2"/>
-    </row>
-    <row r="172">
-      <c r="A172" s="2"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="2"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="2"/>
-    </row>
-    <row r="175">
-      <c r="A175" s="2"/>
-    </row>
-    <row r="176">
-      <c r="A176" s="2"/>
-    </row>
-    <row r="177">
-      <c r="A177" s="2"/>
-    </row>
-    <row r="178">
-      <c r="A178" s="2"/>
-    </row>
-    <row r="179">
-      <c r="A179" s="2"/>
-    </row>
-    <row r="180">
-      <c r="A180" s="2"/>
-    </row>
-    <row r="181">
-      <c r="A181" s="2"/>
-    </row>
-    <row r="182">
-      <c r="A182" s="2"/>
-    </row>
-    <row r="183">
-      <c r="A183" s="2"/>
-    </row>
-    <row r="184">
-      <c r="A184" s="2"/>
-    </row>
-    <row r="185">
-      <c r="A185" s="2"/>
-    </row>
-    <row r="186">
-      <c r="A186" s="2"/>
-    </row>
-    <row r="187">
-      <c r="A187" s="2"/>
-    </row>
-    <row r="189">
-      <c r="A189" s="2"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="2"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="2"/>
-    </row>
-    <row r="192">
-      <c r="A192" s="2"/>
-    </row>
-    <row r="193">
-      <c r="A193" s="2"/>
-    </row>
-    <row r="194">
-      <c r="A194" s="2"/>
-    </row>
-    <row r="195">
-      <c r="A195" s="2"/>
-    </row>
-    <row r="196">
-      <c r="A196" s="2"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="2"/>
-    </row>
-    <row r="198">
-      <c r="A198" s="2"/>
-    </row>
-    <row r="199">
-      <c r="A199" s="2"/>
-    </row>
-    <row r="200">
-      <c r="A200" s="2"/>
-    </row>
-    <row r="201">
-      <c r="A201" s="2"/>
-    </row>
-    <row r="202">
-      <c r="A202" s="2"/>
-    </row>
-    <row r="203">
-      <c r="A203" s="2"/>
-    </row>
-    <row r="204">
-      <c r="A204" s="2"/>
-    </row>
-    <row r="205">
-      <c r="A205" s="2"/>
-    </row>
-    <row r="206">
-      <c r="A206" s="2"/>
-    </row>
-    <row r="207">
-      <c r="A207" s="2"/>
-    </row>
-    <row r="208">
-      <c r="A208" s="2"/>
-    </row>
-    <row r="209">
-      <c r="A209" s="2"/>
-    </row>
-    <row r="210">
-      <c r="A210" s="2"/>
-    </row>
-    <row r="211">
-      <c r="A211" s="2"/>
-    </row>
-    <row r="212">
-      <c r="A212" s="2"/>
-    </row>
-    <row r="213">
-      <c r="A213" s="2"/>
-    </row>
-    <row r="214">
-      <c r="A214" s="2"/>
-    </row>
-    <row r="215">
-      <c r="A215" s="2"/>
-    </row>
-    <row r="216">
-      <c r="A216" s="2"/>
-    </row>
-    <row r="217">
-      <c r="A217" s="2"/>
-    </row>
-    <row r="218">
-      <c r="A218" s="2"/>
-    </row>
-    <row r="219">
-      <c r="A219" s="2"/>
-    </row>
-    <row r="220">
-      <c r="A220" s="2"/>
-    </row>
-    <row r="221">
-      <c r="A221" s="2"/>
-    </row>
-    <row r="222">
-      <c r="A222" s="2"/>
-    </row>
-    <row r="223">
-      <c r="A223" s="2"/>
-    </row>
-    <row r="224">
-      <c r="A224" s="2"/>
-    </row>
-    <row r="225">
-      <c r="A225" s="2"/>
-    </row>
-    <row r="226">
-      <c r="A226" s="2"/>
-    </row>
-    <row r="227">
-      <c r="A227" s="2"/>
-    </row>
-    <row r="228">
-      <c r="A228" s="2"/>
-    </row>
-    <row r="229">
-      <c r="A229" s="2"/>
-    </row>
-    <row r="230">
-      <c r="A230" s="2"/>
-    </row>
-    <row r="231">
-      <c r="A231" s="2"/>
-    </row>
-    <row r="232">
-      <c r="A232" s="2"/>
-    </row>
-    <row r="233">
-      <c r="A233" s="2"/>
-    </row>
-    <row r="234">
-      <c r="A234" s="2"/>
-    </row>
-    <row r="235">
-      <c r="A235" s="2"/>
-    </row>
-    <row r="236">
-      <c r="A236" s="2"/>
-    </row>
-    <row r="237">
-      <c r="A237" s="2"/>
-    </row>
-    <row r="238">
-      <c r="A238" s="2"/>
-    </row>
-    <row r="239">
-      <c r="A239" s="2"/>
-    </row>
-    <row r="240">
-      <c r="A240" s="2"/>
-    </row>
-    <row r="241">
-      <c r="A241" s="2"/>
-    </row>
-    <row r="242">
-      <c r="A242" s="2"/>
-    </row>
-    <row r="243">
-      <c r="A243" s="2"/>
-    </row>
-    <row r="244">
-      <c r="A244" s="2"/>
-    </row>
-    <row r="245">
-      <c r="A245" s="2"/>
-    </row>
-    <row r="246">
-      <c r="A246" s="2"/>
-    </row>
-    <row r="247">
-      <c r="A247" s="2"/>
-    </row>
-    <row r="248">
-      <c r="A248" s="2"/>
-    </row>
-    <row r="249">
-      <c r="A249" s="2"/>
-    </row>
-    <row r="250">
-      <c r="A250" s="2"/>
-    </row>
-    <row r="251">
-      <c r="A251" s="2"/>
-    </row>
-    <row r="252">
-      <c r="A252" s="2"/>
-    </row>
-    <row r="253">
-      <c r="A253" s="2"/>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2">
-        <v>44544.0</v>
+        <v>44557</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>44535.0</v>
+        <v>44546</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>44514.0</v>
+        <v>44539</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>44494.0</v>
+        <v>44535</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2"/>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2">
-        <v>44557.0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
-        <v>44546.0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>44539.0</v>
-      </c>
-      <c r="B3" s="3" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>44535.0</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>44524.0</v>
+        <v>44524</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>44515.0</v>
+        <v>44515</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>44500.0</v>
+        <v>44500</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>44492.0</v>
+        <v>44492</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <v>44486.0</v>
+        <v>44486</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <v>44483.0</v>
+        <v>44483</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2">
-        <v>44482.0</v>
+        <v>44482</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2">
-        <v>44480.0</v>
+        <v>44480</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2">
-        <v>44479.0</v>
+        <v>44479</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2">
-        <v>44478.0</v>
+        <v>44478</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15">
@@ -8548,6 +7944,9 @@
       <c r="A34" s="2"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>